<commit_message>
Código para criar plainilha update_cards.xlsx gerada
</commit_message>
<xml_diff>
--- a/jira_cards.xlsx
+++ b/jira_cards.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G111"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,7 +518,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>A Produzir</t>
+          <t>Liberado Engenharia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>A Produzir</t>
+          <t>Liberado Engenharia</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -619,32 +619,32 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/TENSYLON-752</t>
+          <t>https://carboncars.atlassian.net/browse/TENSYLON-730</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>30580</t>
+          <t>30483</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Liberado Engenharia</t>
+          <t>A Produzir</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AUDI - SQ6 E-TRON SPORTBACK - 2025</t>
+          <t>JEEP - COMMANDER SUV - 2026</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>11/03/2026</t>
         </is>
       </c>
     </row>
@@ -656,17 +656,17 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/TENSYLON-746</t>
+          <t>https://carboncars.atlassian.net/browse/TENSYLON-728</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>30538</t>
+          <t>30472</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Liberado Engenharia</t>
+          <t>A Produzir</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -676,12 +676,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PORSCHE - 911 - 2025</t>
+          <t>LAND ROVER - DISCOVERY SPORT SUV - 2023</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
@@ -693,91 +693,81 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/TENSYLON-730</t>
+          <t>https://carboncars.atlassian.net/browse/TENSYLON-674</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>30483</t>
+          <t>30281</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>A Produzir</t>
+          <t>Liberado Engenharia</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>JEEP - COMMANDER SUV - 2026</t>
+          <t>MERCEDES-BENZ - GLS SUV - 2026</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tensylon</t>
+          <t>Manta</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/TENSYLON-728</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30807</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>30472</t>
+          <t>30439 PEDIDO AVULSO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>A Produzir</t>
+          <t>Liberado Engenharia</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>🟢RECEBIDO LIBERADO</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>LAND ROVER - DISCOVERY SPORT SUV - 2023</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>09/03/2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tensylon</t>
+          <t>Manta</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/TENSYLON-691</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30781</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>30351</t>
+          <t>30911 PED AVULSO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Liberado Engenharia</t>
+          <t>A Produzir</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -787,29 +777,24 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>GWM - HAVAL H9 SUV - 2026</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>09/03/2026</t>
+          <t>VOLVO - XC90 - 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tensylon</t>
+          <t>Manta</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/TENSYLON-674</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30763</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>30281</t>
+          <t>31136 - ALT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -819,17 +804,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ - GLS SUV - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -841,12 +826,12 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30763</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30740</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>31136 - ALT</t>
+          <t>31140</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -878,12 +863,12 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30740</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30739</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>31140</t>
+          <t>31139</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -915,12 +900,12 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30739</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30738</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>31139</t>
+          <t>31138</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -952,12 +937,12 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30738</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30737</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>31138</t>
+          <t>31137</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -989,12 +974,12 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30737</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30735</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>31137</t>
+          <t>31135</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1026,17 +1011,17 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30735</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30734</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>31135</t>
+          <t>31134</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Liberado Engenharia</t>
+          <t>A Produzir</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1051,7 +1036,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
@@ -1063,17 +1048,17 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30734</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30733</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>31134</t>
+          <t>31133</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>A Produzir</t>
+          <t>Liberado Engenharia</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1088,7 +1073,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1085,12 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30733</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30732</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>31133</t>
+          <t>31132</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1120,7 +1105,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1137,12 +1122,12 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30732</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30730</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>31132</t>
+          <t>31130</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1174,12 +1159,12 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30730</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30720</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>31130</t>
+          <t>30931 - ALT</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1189,7 +1174,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1211,12 +1196,12 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30720</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30718</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>30931 - ALT</t>
+          <t>31120</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1226,7 +1211,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1248,12 +1233,12 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30718</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30658</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>31120</t>
+          <t>31061</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1285,12 +1270,12 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30658</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30657</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>31061</t>
+          <t>31060</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1322,12 +1307,12 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30657</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30656</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>31060</t>
+          <t>31059</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1359,12 +1344,12 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30656</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30649</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>31059</t>
+          <t>31054</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1379,7 +1364,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1396,12 +1381,12 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30649</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30647</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>31054</t>
+          <t>31052</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1416,12 +1401,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>JEEP - COMPASS SUV - 2026</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
@@ -1433,12 +1418,12 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30647</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30638</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>31052</t>
+          <t>31043</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1453,7 +1438,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>JEEP - COMPASS SUV - 2026</t>
+          <t>GWM - HAVAL H6 PHEV 19 - 2026</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1470,12 +1455,12 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30638</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30630</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>31043</t>
+          <t>31036</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1490,7 +1475,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>GWM - HAVAL H6 PHEV 19 - 2026</t>
+          <t>GWM - HAVAL H6 GT - 2026</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1507,12 +1492,12 @@
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30630</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30628</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>31036</t>
+          <t>31034</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1527,7 +1512,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>GWM - HAVAL H6 GT - 2026</t>
+          <t>GWM - HAVAL H9 SUV - 2026</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1544,12 +1529,12 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30628</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30624</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>31034</t>
+          <t>31030</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1564,12 +1549,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>GWM - HAVAL H9 SUV - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -1581,12 +1566,12 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30624</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30622</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>31030</t>
+          <t>31028</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1596,7 +1581,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1618,12 +1603,12 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30622</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30619</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>31028</t>
+          <t>31025</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1633,7 +1618,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1655,12 +1640,12 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30619</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30615</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>31025</t>
+          <t>31021</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1670,12 +1655,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1692,12 +1677,12 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30615</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30613</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>31021</t>
+          <t>31019</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1729,12 +1714,12 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30613</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30610</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>31019</t>
+          <t>31016</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1744,7 +1729,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1766,12 +1751,12 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30610</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30609</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>31016</t>
+          <t>31015</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1781,7 +1766,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1803,12 +1788,12 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30609</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30608</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>31015</t>
+          <t>31014</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1840,12 +1825,12 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30608</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30607</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>31014</t>
+          <t>31013</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1860,7 +1845,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1877,12 +1862,12 @@
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30607</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30606</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>31013</t>
+          <t>31012</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1897,7 +1882,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1914,12 +1899,12 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30606</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30602</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>31012</t>
+          <t>31009</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1951,12 +1936,12 @@
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30602</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30600</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>31009</t>
+          <t>31006</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1988,12 +1973,12 @@
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30600</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30597</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>31006</t>
+          <t>31003</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2025,12 +2010,12 @@
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30597</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30595</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>31003</t>
+          <t>31001</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2045,7 +2030,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2062,12 +2047,12 @@
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30595</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30594</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>31001</t>
+          <t>31000</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2077,7 +2062,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2099,12 +2084,12 @@
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30594</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30593</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>31000</t>
+          <t>30999</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2114,7 +2099,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2136,12 +2121,12 @@
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30593</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30590</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>30999</t>
+          <t>30996</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2151,7 +2136,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2173,12 +2158,12 @@
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30590</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30589</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>30996</t>
+          <t>30995</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2188,12 +2173,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2210,12 +2195,12 @@
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30589</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30588</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>30995</t>
+          <t>30994</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2247,12 +2232,12 @@
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30588</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30586</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>30994</t>
+          <t>30992</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2284,12 +2269,12 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30586</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30585</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>30992</t>
+          <t>30991</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2321,12 +2306,12 @@
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30585</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30584</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>30991</t>
+          <t>30990</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2341,7 +2326,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2358,12 +2343,12 @@
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30584</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30583</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>30990</t>
+          <t>30989</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2395,12 +2380,12 @@
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30583</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30582</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>30989</t>
+          <t>30988</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2432,12 +2417,12 @@
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30582</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30581</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>30988</t>
+          <t>30987</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2469,12 +2454,12 @@
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30581</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30580</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>30987</t>
+          <t>30986</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2506,12 +2491,12 @@
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30580</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30579</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>30986</t>
+          <t>30985</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2543,12 +2528,12 @@
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30579</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30578</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>30985</t>
+          <t>30984</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2580,12 +2565,12 @@
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30578</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30577</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>30984</t>
+          <t>30983</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2617,12 +2602,12 @@
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30577</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30576</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>30983</t>
+          <t>30982</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2654,12 +2639,12 @@
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30576</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30575</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>30982</t>
+          <t>30981</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2691,12 +2676,12 @@
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30575</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30574</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>30981</t>
+          <t>30980</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2711,7 +2696,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2728,12 +2713,12 @@
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30574</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30573</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>30980</t>
+          <t>30979</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2765,12 +2750,12 @@
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30573</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30571</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>30979</t>
+          <t>30977</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2785,7 +2770,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2802,12 +2787,12 @@
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30571</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30570</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>30977</t>
+          <t>30976</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2839,12 +2824,12 @@
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30570</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30569</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>30976</t>
+          <t>30975</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2876,12 +2861,12 @@
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30569</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30568</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>30975</t>
+          <t>30974</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2891,17 +2876,17 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>HONDA - WR-V - 2026</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
@@ -2913,12 +2898,12 @@
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30568</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30567</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>30974</t>
+          <t>30973</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2933,7 +2918,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>HONDA - WR-V - 2026</t>
+          <t>HONDA - NEW HR-V SUV - 2026</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2950,12 +2935,12 @@
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30567</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30542</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>30973</t>
+          <t>30948</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2970,7 +2955,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>HONDA - NEW HR-V SUV - 2026</t>
+          <t>BMW - X3 SUV - 2026</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2987,12 +2972,12 @@
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30542</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30530</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>30948</t>
+          <t>30939</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3007,12 +2992,12 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>BMW - X3 SUV - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -3024,12 +3009,12 @@
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30530</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30526</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>30939</t>
+          <t>30935</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3039,17 +3024,17 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
@@ -3061,12 +3046,12 @@
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30526</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30525</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>30935</t>
+          <t>30934</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3098,12 +3083,12 @@
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30525</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30523</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>30934</t>
+          <t>30932</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3135,12 +3120,12 @@
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30523</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30521</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>30932</t>
+          <t>30930</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3155,12 +3140,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -3172,12 +3157,12 @@
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30521</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30515</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>30930</t>
+          <t>30924</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3209,12 +3194,12 @@
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30515</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30514</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>30924</t>
+          <t>30923</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3246,12 +3231,12 @@
       </c>
       <c r="B77" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30514</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30513</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>30923</t>
+          <t>30922</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3266,7 +3251,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3283,12 +3268,12 @@
       </c>
       <c r="B78" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30513</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30512</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>30922</t>
+          <t>30921</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3308,7 +3293,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -3320,12 +3305,12 @@
       </c>
       <c r="B79" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30512</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30511</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>30921</t>
+          <t>30920</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3357,12 +3342,12 @@
       </c>
       <c r="B80" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30511</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30510</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>30920</t>
+          <t>30919</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3377,12 +3362,12 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -3394,12 +3379,12 @@
       </c>
       <c r="B81" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30510</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30509</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>30919</t>
+          <t>30918</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3409,7 +3394,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3431,12 +3416,12 @@
       </c>
       <c r="B82" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30509</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30507</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>30918</t>
+          <t>30916</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3446,7 +3431,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3468,12 +3453,12 @@
       </c>
       <c r="B83" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30507</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30506</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>30916</t>
+          <t>30915</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3505,12 +3490,12 @@
       </c>
       <c r="B84" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30506</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30505</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>30915</t>
+          <t>30914</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3542,12 +3527,12 @@
       </c>
       <c r="B85" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30505</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30504</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>30914</t>
+          <t>30913</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3557,17 +3542,17 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>JAECOO - JAECOO 7 SUV - 2026</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
@@ -3579,12 +3564,12 @@
       </c>
       <c r="B86" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30504</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30479</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>30913</t>
+          <t>30892</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3599,7 +3584,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>JAECOO - JAECOO 7 SUV - 2026</t>
+          <t>LEXUS - NX 350 H SUV - 2026</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -3616,12 +3601,12 @@
       </c>
       <c r="B87" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30479</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30469</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>30892</t>
+          <t>30882</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3636,7 +3621,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>LEXUS - NX 350 H SUV - 2026</t>
+          <t>MINI - COOPER 04 PORTAS HATCH - 2026</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -3653,12 +3638,12 @@
       </c>
       <c r="B88" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30469</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30464</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>30882</t>
+          <t>30877</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3668,17 +3653,17 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>MINI - COOPER 04 PORTAS HATCH - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -3690,12 +3675,12 @@
       </c>
       <c r="B89" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30464</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30463</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>30877</t>
+          <t>30876</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3710,7 +3695,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -3727,12 +3712,12 @@
       </c>
       <c r="B90" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30463</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30462</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>30876</t>
+          <t>30875</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -3747,7 +3732,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -3764,12 +3749,12 @@
       </c>
       <c r="B91" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30462</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30452</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>30875</t>
+          <t>30865</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3779,7 +3764,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3801,12 +3786,12 @@
       </c>
       <c r="B92" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30452</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30451</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>30865</t>
+          <t>30864</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3821,12 +3806,12 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>KIA - CARNIVAL VAN - 2025</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
@@ -3838,12 +3823,12 @@
       </c>
       <c r="B93" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30451</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30428</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>30864</t>
+          <t>30841</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3853,17 +3838,17 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>KIA - CARNIVAL VAN - 2025</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -3875,12 +3860,12 @@
       </c>
       <c r="B94" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30428</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30421</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>30841</t>
+          <t>30834</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3912,12 +3897,12 @@
       </c>
       <c r="B95" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30421</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30420</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>30834</t>
+          <t>30833</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -3949,12 +3934,12 @@
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30420</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30367</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>30833</t>
+          <t>30786</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3974,7 +3959,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -3986,12 +3971,12 @@
       </c>
       <c r="B97" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30367</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30309</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>30786</t>
+          <t>30735</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4006,12 +3991,12 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - SW4 SUV - 2026</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
@@ -4023,12 +4008,12 @@
       </c>
       <c r="B98" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30309</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30257</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>30735</t>
+          <t>30687</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4038,7 +4023,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4048,7 +4033,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -4060,12 +4045,12 @@
       </c>
       <c r="B99" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30257</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30242</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>30687</t>
+          <t>30674</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -4075,17 +4060,17 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>TOYOTA - SW4 SUV - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
@@ -4097,12 +4082,12 @@
       </c>
       <c r="B100" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30242</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30224</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>30674</t>
+          <t>30657</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -4112,17 +4097,17 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - SW4 SUV - 2026</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -4134,12 +4119,12 @@
       </c>
       <c r="B101" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30224</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30196</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>30657</t>
+          <t>30632</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4149,17 +4134,17 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>TOYOTA - SW4 SUV - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
@@ -4171,12 +4156,12 @@
       </c>
       <c r="B102" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30196</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30191</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>30632</t>
+          <t>30628</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -4186,17 +4171,17 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>BMW - X3 SUV - 2026</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
@@ -4208,17 +4193,17 @@
       </c>
       <c r="B103" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30191</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30026</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>30628</t>
+          <t>30483</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>A Produzir</t>
+          <t>Liberado Engenharia</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4228,7 +4213,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>BMW - X3 SUV - 2026</t>
+          <t>JEEP - COMMANDER SUV - 2026</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -4245,12 +4230,12 @@
       </c>
       <c r="B104" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30026</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29945</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>30483</t>
+          <t>30412</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -4265,7 +4250,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>JEEP - COMMANDER SUV - 2026</t>
+          <t>GWM - HAVAL H6 HEV 2 - 2026</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -4282,17 +4267,17 @@
       </c>
       <c r="B105" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30013</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29923</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>30472</t>
+          <t>30392</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>A Produzir</t>
+          <t>Liberado Engenharia</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4302,12 +4287,12 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>LAND ROVER - DISCOVERY SPORT SUV - 2023</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -4319,12 +4304,12 @@
       </c>
       <c r="B106" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29945</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29866</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>30412</t>
+          <t>30344</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -4339,12 +4324,12 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>GWM - HAVAL H6 HEV 2 - 2026</t>
+          <t>LAND ROVER - DISCOVERY METROPOLITAN - 2024</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
@@ -4356,12 +4341,12 @@
       </c>
       <c r="B107" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29923</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29791</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>30392</t>
+          <t>30281</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -4376,12 +4361,12 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>MERCEDES-BENZ - GLS SUV - 2026</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
@@ -4393,12 +4378,12 @@
       </c>
       <c r="B108" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29866</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29372</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>30344</t>
+          <t>29901</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -4408,12 +4393,12 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>LAND ROVER - DISCOVERY METROPOLITAN - 2024</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -4430,12 +4415,12 @@
       </c>
       <c r="B109" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29791</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-27100</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>30281</t>
+          <t>28192</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -4445,89 +4430,15 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ - GLS SUV - 2026</t>
+          <t>LEXUS - RX 500H SUV - 2025</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
-        <is>
-          <t>10/03/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>Manta</t>
-        </is>
-      </c>
-      <c r="B110" s="1" t="inlineStr">
-        <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29372</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>29901</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>Liberado Engenharia</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>🟢RECEBIDO LIBERADO</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>13/03/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>Manta</t>
-        </is>
-      </c>
-      <c r="B111" s="1" t="inlineStr">
-        <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-27100</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>28192</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>Liberado Engenharia</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>LEXUS - RX 500H SUV - 2025</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
         <is>
           <t>10/03/2026</t>
         </is>
@@ -4643,8 +4554,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B107" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B108" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId110"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>